<commit_message>
docs(bom): Steckerbezeichnungen angepasst und LiPo-Akku zugefügt
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/KiCAD-PCB/Version20251022/BOM_ESP32C6_gasometer.xlsx
+++ b/KiCAD-PCB/Version20251022/BOM_ESP32C6_gasometer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\gas-o-meter2\KiCAD-PCB\Version20251022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C11357-0740-4116-AF0E-1CE375BC4E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FE68F77-0520-468B-AD5C-36804B2C982A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="25650" windowHeight="14520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="645" windowWidth="25650" windowHeight="14520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_ESP32C6_gasometer" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
   <si>
     <t>Reference</t>
   </si>
@@ -103,22 +103,28 @@
     <t>J3</t>
   </si>
   <si>
-    <t>JST-Conn. / Battery Connector</t>
-  </si>
-  <si>
     <t>KSK-1A87-1520</t>
   </si>
   <si>
     <t>Generic connector, single row, 01x02 // Reed</t>
   </si>
   <si>
-    <t>JST-SH 1.25 2pin plug/socket</t>
-  </si>
-  <si>
     <t>Generic connector, single row, 01x02 // Batterie</t>
   </si>
   <si>
     <t>JST-PH 2.00 2pin socket</t>
+  </si>
+  <si>
+    <t>Li-Polymer Battery  52x34x5,0mm</t>
+  </si>
+  <si>
+    <t>LiPo 1000mAh 523450</t>
+  </si>
+  <si>
+    <t>JST-XH 1.25 2pin socket</t>
+  </si>
+  <si>
+    <t>JST-XH 1.25 2pin plug</t>
   </si>
 </sst>
 </file>
@@ -479,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -514,10 +520,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -528,10 +534,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -573,7 +579,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -628,8 +634,25 @@
       <c r="A10" t="s">
         <v>25</v>
       </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>